<commit_message>
feat(270): Cambio de títulos en plantilla de animales
</commit_message>
<xml_diff>
--- a/templates/template_import_data_animals.xlsx
+++ b/templates/template_import_data_animals.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DescargasNavegador\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\source\repos\GanSoft\gansoft-resx\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD34E7CB-9740-4474-80E7-38925ABCE81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16815" windowHeight="8925"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Animales" sheetId="1" r:id="rId1"/>
@@ -77,12 +78,6 @@
     <t>Uso Frecuente</t>
   </si>
   <si>
-    <t>Dósis</t>
-  </si>
-  <si>
-    <t>Edad</t>
-  </si>
-  <si>
     <t>Causa de Entrada</t>
   </si>
   <si>
@@ -96,12 +91,18 @@
   </si>
   <si>
     <t>Próxima Revisión</t>
+  </si>
+  <si>
+    <t>Edad de embrión</t>
+  </si>
+  <si>
+    <t>Dósis semen o embrión</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -152,13 +153,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -173,28 +173,28 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -221,7 +221,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -269,33 +269,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Animales" displayName="Animales" ref="A1:X11" totalsRowShown="0" headerRowDxfId="24">
-  <autoFilter ref="A1:X11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:X11" totalsRowShown="0" headerRowDxfId="24">
+  <autoFilter ref="A1:X11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="24">
-    <tableColumn id="1" name="Práctico" dataDxfId="23"/>
-    <tableColumn id="2" name="Único" dataDxfId="22"/>
-    <tableColumn id="3" name="Categoría" dataDxfId="21"/>
-    <tableColumn id="4" name="Estatus" dataDxfId="20"/>
-    <tableColumn id="5" name="Lote" dataDxfId="19"/>
-    <tableColumn id="6" name="Fecha de Entrada" dataDxfId="18"/>
-    <tableColumn id="7" name="Causa de Entrada" dataDxfId="17"/>
-    <tableColumn id="8" name="Técnico" dataDxfId="16"/>
-    <tableColumn id="9" name="Comentario" dataDxfId="15"/>
-    <tableColumn id="10" name="Uso Frecuente" dataDxfId="14"/>
-    <tableColumn id="11" name="Dósis" dataDxfId="13"/>
-    <tableColumn id="12" name="Edad" dataDxfId="12"/>
-    <tableColumn id="13" name="Estatus Reproductivo" dataDxfId="11"/>
-    <tableColumn id="14" name="Estatus Productivo" dataDxfId="10"/>
-    <tableColumn id="15" name="Próxima Revisión" dataDxfId="9"/>
-    <tableColumn id="16" name="ID Electrónico" dataDxfId="8"/>
-    <tableColumn id="17" name="Nombre" dataDxfId="7"/>
-    <tableColumn id="18" name="Propietario" dataDxfId="6"/>
-    <tableColumn id="19" name="Padre" dataDxfId="5"/>
-    <tableColumn id="20" name="Madre" dataDxfId="4"/>
-    <tableColumn id="21" name="Composición Racial" dataDxfId="3"/>
-    <tableColumn id="22" name="Fecha de Nacimiento" dataDxfId="2"/>
-    <tableColumn id="23" name="Color" dataDxfId="1"/>
-    <tableColumn id="24" name="Clasificación" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Práctico" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Único" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Categoría" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Estatus" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Lote" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Fecha de Entrada" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Causa de Entrada" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Técnico" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Comentario" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Uso Frecuente" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Dósis semen o embrión" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Edad de embrión" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Estatus Reproductivo" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Estatus Productivo" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Próxima Revisión" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="ID Electrónico" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Nombre" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Propietario" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Padre" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Madre" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Composición Racial" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Fecha de Nacimiento" dataDxfId="2"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Color" dataDxfId="1"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Clasificación" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -563,9 +563,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
@@ -576,6 +576,8 @@
     <col min="8" max="8" width="12.85546875" customWidth="1"/>
     <col min="9" max="9" width="15.5703125" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.28515625" customWidth="1"/>
     <col min="14" max="14" width="19.42578125" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
@@ -589,27 +591,27 @@
     <col min="24" max="24" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>19</v>
+      <c r="F1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -621,19 +623,19 @@
         <v>16</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>7</v>
@@ -929,22 +931,22 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Hembra Lactante,Hembra Destetada,Hembra Adulta,Hembra Madura,Macho Lactante,Macho Destetado,Macho Adulto,Macho Maduro,Semen,Embrión"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D11" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Activo,Inactivo,Referencia"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G11" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Nacimiento,Compra,Ingreso"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J11" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M11" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Vacía,Preñada,En espera"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N11" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Criando,Ordeño,Seca"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Merged PR 1162: Cambio de títulos en plantilla de animales
feat(270): Cambio de títulos en plantilla de animales

Related work items: #270
</commit_message>
<xml_diff>
--- a/templates/template_import_data_animals.xlsx
+++ b/templates/template_import_data_animals.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DescargasNavegador\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\source\repos\GanSoft\gansoft-resx\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD34E7CB-9740-4474-80E7-38925ABCE81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16815" windowHeight="8925"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Animales" sheetId="1" r:id="rId1"/>
@@ -77,12 +78,6 @@
     <t>Uso Frecuente</t>
   </si>
   <si>
-    <t>Dósis</t>
-  </si>
-  <si>
-    <t>Edad</t>
-  </si>
-  <si>
     <t>Causa de Entrada</t>
   </si>
   <si>
@@ -96,12 +91,18 @@
   </si>
   <si>
     <t>Próxima Revisión</t>
+  </si>
+  <si>
+    <t>Edad de embrión</t>
+  </si>
+  <si>
+    <t>Dósis semen o embrión</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -152,13 +153,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -173,28 +173,28 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -221,7 +221,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -269,33 +269,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Animales" displayName="Animales" ref="A1:X11" totalsRowShown="0" headerRowDxfId="24">
-  <autoFilter ref="A1:X11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Animales" displayName="Animales" ref="A1:X11" totalsRowShown="0" headerRowDxfId="24">
+  <autoFilter ref="A1:X11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="24">
-    <tableColumn id="1" name="Práctico" dataDxfId="23"/>
-    <tableColumn id="2" name="Único" dataDxfId="22"/>
-    <tableColumn id="3" name="Categoría" dataDxfId="21"/>
-    <tableColumn id="4" name="Estatus" dataDxfId="20"/>
-    <tableColumn id="5" name="Lote" dataDxfId="19"/>
-    <tableColumn id="6" name="Fecha de Entrada" dataDxfId="18"/>
-    <tableColumn id="7" name="Causa de Entrada" dataDxfId="17"/>
-    <tableColumn id="8" name="Técnico" dataDxfId="16"/>
-    <tableColumn id="9" name="Comentario" dataDxfId="15"/>
-    <tableColumn id="10" name="Uso Frecuente" dataDxfId="14"/>
-    <tableColumn id="11" name="Dósis" dataDxfId="13"/>
-    <tableColumn id="12" name="Edad" dataDxfId="12"/>
-    <tableColumn id="13" name="Estatus Reproductivo" dataDxfId="11"/>
-    <tableColumn id="14" name="Estatus Productivo" dataDxfId="10"/>
-    <tableColumn id="15" name="Próxima Revisión" dataDxfId="9"/>
-    <tableColumn id="16" name="ID Electrónico" dataDxfId="8"/>
-    <tableColumn id="17" name="Nombre" dataDxfId="7"/>
-    <tableColumn id="18" name="Propietario" dataDxfId="6"/>
-    <tableColumn id="19" name="Padre" dataDxfId="5"/>
-    <tableColumn id="20" name="Madre" dataDxfId="4"/>
-    <tableColumn id="21" name="Composición Racial" dataDxfId="3"/>
-    <tableColumn id="22" name="Fecha de Nacimiento" dataDxfId="2"/>
-    <tableColumn id="23" name="Color" dataDxfId="1"/>
-    <tableColumn id="24" name="Clasificación" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Práctico" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Único" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Categoría" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Estatus" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Lote" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Fecha de Entrada" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Causa de Entrada" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Técnico" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Comentario" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Uso Frecuente" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Dósis semen o embrión" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Edad de embrión" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Estatus Reproductivo" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Estatus Productivo" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Próxima Revisión" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="ID Electrónico" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Nombre" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Propietario" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Padre" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Madre" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Composición Racial" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Fecha de Nacimiento" dataDxfId="2"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Color" dataDxfId="1"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Clasificación" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -563,9 +563,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
@@ -576,6 +576,8 @@
     <col min="8" max="8" width="12.85546875" customWidth="1"/>
     <col min="9" max="9" width="15.5703125" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.28515625" customWidth="1"/>
     <col min="14" max="14" width="19.42578125" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
@@ -589,27 +591,27 @@
     <col min="24" max="24" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>19</v>
+      <c r="F1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -621,19 +623,19 @@
         <v>16</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>7</v>
@@ -929,22 +931,22 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Hembra Lactante,Hembra Destetada,Hembra Adulta,Hembra Madura,Macho Lactante,Macho Destetado,Macho Adulto,Macho Maduro,Semen,Embrión"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D11" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Activo,Inactivo,Referencia"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G11" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Nacimiento,Compra,Ingreso"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J11" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M11" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Vacía,Preñada,En espera"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N11" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Criando,Ordeño,Seca"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>